<commit_message>
Added datasets to QGIS & formatted basics
</commit_message>
<xml_diff>
--- a/Data Catalog.xlsx
+++ b/Data Catalog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John\Documents\hillsborogis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FFE81CA-EEEC-4E2B-B1A9-162B82212A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{587D5D03-3DA4-4CE3-A304-58DC9B3D1182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="datasets" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,19 @@
     <sheet name="relationships" sheetId="3" r:id="rId3"/>
     <sheet name="analysis log" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="+kIrob3A2t3jj/CNQOp5cw4gPnP5+XCJiZ4+LTmjP0I="/>
     </ext>
@@ -31044,9 +31055,9 @@
   <dimension ref="A1:E1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.42578125" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.42578125" customWidth="1"/>
     <col min="5" max="5" width="80.85546875" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" customWidth="1"/>
@@ -32294,6 +32305,7 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>